<commit_message>
changing the course description into table format
</commit_message>
<xml_diff>
--- a/media/bookings/course_bookings.xlsx
+++ b/media/bookings/course_bookings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -841,6 +841,59 @@
       <c r="K8" t="inlineStr">
         <is>
           <t>23-02-2026 21:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Shobana V</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>shobavelu1424@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>9626554049</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Full Stack Development (Example – Dynamic Based on Selection)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>4999</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>31-05-2026 20:49</t>
         </is>
       </c>
     </row>

</xml_diff>